<commit_message>
testing menggunakan data baru 2026
</commit_message>
<xml_diff>
--- a/output/evaluation_report/databaru_top_rules_evaluation_70_30.xlsx
+++ b/output/evaluation_report/databaru_top_rules_evaluation_70_30.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,11 +457,6 @@
           <t>Kategori Rule</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Status Pengujian</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -494,11 +489,6 @@
           <t>Strong Pattern</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Konsisten</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -531,11 +521,6 @@
           <t>Strong Pattern</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Konsisten</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -568,11 +553,6 @@
           <t>Strong Pattern</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Konsisten</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -605,11 +585,6 @@
           <t>Strong Pattern</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Konsisten</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -642,11 +617,6 @@
           <t>Strong Pattern</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Konsisten</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -679,11 +649,6 @@
           <t>Moderate Pattern</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Konsisten</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -716,11 +681,6 @@
           <t>Moderate Pattern</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Konsisten</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -753,11 +713,6 @@
           <t>Moderate Pattern</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Konsisten</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -790,11 +745,6 @@
           <t>Moderate Pattern</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Konsisten</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -825,11 +775,6 @@
       <c r="H11" t="inlineStr">
         <is>
           <t>Moderate Pattern</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Konsisten</t>
         </is>
       </c>
     </row>

</xml_diff>